<commit_message>
#204 Add support for CSV and XLSX formats for input tables
</commit_message>
<xml_diff>
--- a/13_csa/rscript/tests/data/sulsel/tabel_acuan_konversi.xlsx
+++ b/13_csa/rscript/tests/data/sulsel/tabel_acuan_konversi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ICRAF\Kodingan\icraf-indonesia\lumens-shiny\13_csa\rscript\tests\data\sulsel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{58D75C5A-145F-485F-A06E-278279E8F87F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{601861E9-C1F0-4AA9-B9E5-213DCE367E6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9C254F7A-495D-440E-9E5F-3020018E4D4B}"/>
   </bookViews>
@@ -46,9 +46,6 @@
     <t>Tidak ditanami padi</t>
   </si>
   <si>
-    <t>N Urea</t>
-  </si>
-  <si>
     <t>N NPK 15-10-12</t>
   </si>
   <si>
@@ -106,9 +103,6 @@
     <t>GWP N2O</t>
   </si>
   <si>
-    <t>N_Urea</t>
-  </si>
-  <si>
     <t>N_NPK</t>
   </si>
   <si>
@@ -197,6 +191,12 @@
   </si>
   <si>
     <t>Faktor Emisi CH4 per luas panen</t>
+  </si>
+  <si>
+    <t>N UREA</t>
+  </si>
+  <si>
+    <t>N_UREA</t>
   </si>
 </sst>
 </file>
@@ -680,9 +680,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="42">
@@ -1062,18 +1060,16 @@
   <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="2"/>
-    <col min="2" max="2" width="23.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>24</v>
+      <c r="A1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -1081,371 +1077,371 @@
       <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>49</v>
+      <c r="E1" t="s">
+        <v>47</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D2">
         <v>6.3899999999999998E-2</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>38</v>
+      <c r="E2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
+      <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D3">
         <v>0.90249999999999997</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>56</v>
+      <c r="E3" t="s">
+        <v>54</v>
       </c>
       <c r="F3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+      <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D4">
         <v>3.3599999999999998E-2</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>56</v>
+      <c r="E4" t="s">
+        <v>54</v>
       </c>
       <c r="F4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D5">
         <v>15635</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>41</v>
+      <c r="E5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F5" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
+      <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D6">
         <v>173243</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>57</v>
+      <c r="E6" t="s">
+        <v>55</v>
       </c>
       <c r="F6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
+      <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D7">
         <v>403316</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
         <v>57</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="2">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>8</v>
-      </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="D8">
         <v>0.46</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>56</v>
+      <c r="E8" t="s">
+        <v>54</v>
       </c>
       <c r="F8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
+      <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>9</v>
+      <c r="B9" t="s">
+        <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D9">
         <v>0.15</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>47</v>
+      <c r="E9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="2">
+      <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>25</v>
+      <c r="B10" t="s">
+        <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>56</v>
+      <c r="E10" t="s">
+        <v>54</v>
       </c>
       <c r="F10" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
+      <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>26</v>
+      <c r="B11" t="s">
+        <v>25</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D11">
         <v>27.2</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>46</v>
+      <c r="E11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="2">
+      <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>27</v>
+      <c r="B12" t="s">
+        <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D12">
         <v>273</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>46</v>
+      <c r="E12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="2">
+      <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>44</v>
+      <c r="B13" t="s">
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D13">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>47</v>
+      <c r="E13" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="2">
+      <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>45</v>
+      <c r="B14" t="s">
+        <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D14">
         <v>0.2</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
         <v>56</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="2">
+      <c r="C15" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15">
+        <v>1.61</v>
+      </c>
+      <c r="E15" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16">
         <v>15</v>
       </c>
-      <c r="D15" s="1">
-        <v>1.61</v>
-      </c>
-      <c r="E15" s="2" t="s">
+      <c r="B16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
+        <v>54</v>
+      </c>
+      <c r="F16" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="s">
+        <v>54</v>
+      </c>
+      <c r="F17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" t="s">
+        <v>54</v>
+      </c>
+      <c r="F18" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>240</v>
+      </c>
+      <c r="E19" t="s">
+        <v>49</v>
+      </c>
+      <c r="F19" t="s">
         <v>50</v>
-      </c>
-      <c r="F15" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="2">
-        <v>15</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16" s="1">
-        <v>1</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F16" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="2">
-        <v>16</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D17" s="1">
-        <v>1</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F17" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="2">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D18" s="1">
-        <v>1</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F18" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="2">
-        <v>18</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D19" s="1">
-        <v>240</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F19" t="s">
-        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>